<commit_message>
Nueva revesión delos modelos
</commit_message>
<xml_diff>
--- a/data/external/dr_ESdEadulto_2023.xlsx
+++ b/data/external/dr_ESdEadulto_2023.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="14160" windowHeight="12300" activeTab="1"/>
+    <workbookView windowWidth="15945" windowHeight="12300"/>
   </bookViews>
   <sheets>
     <sheet name="Diseño" sheetId="22" r:id="rId1"/>
@@ -6419,7 +6419,7 @@
     <numFmt numFmtId="178" formatCode="_ * #.##0_ ;_ * \-#.##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_(\$* #.##0_);_(\$* \(#.##0\);_(\$* &quot;-&quot;_);_(@_)"/>
   </numFmts>
-  <fonts count="46">
+  <fonts count="44">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -6427,11 +6427,6 @@
     </font>
     <font>
       <sz val="12"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <name val="Arial"/>
       <charset val="134"/>
     </font>
@@ -6467,12 +6462,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <b/>
       <sz val="10"/>
       <color indexed="8"/>
@@ -6495,6 +6484,13 @@
     <font>
       <sz val="10"/>
       <color indexed="10"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF800080"/>
       <name val="Arial"/>
       <charset val="134"/>
     </font>
@@ -6545,13 +6541,6 @@
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="10"/>
-      <color rgb="FF800080"/>
-      <name val="Arial"/>
-      <charset val="134"/>
     </font>
     <font>
       <b/>
@@ -6734,7 +6723,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="39">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -6828,12 +6817,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -7275,156 +7258,156 @@
   </borders>
   <cellStyleXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="23" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="23" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="23" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="23" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="178" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="23" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="179" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="19" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="19" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="9" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="10" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="9" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="10" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="10" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="11" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="10" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="11" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="26" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="35" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="26" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="36" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="37" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="163">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -7432,425 +7415,425 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="6"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="6" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="50"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="50" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="50" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="50" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="50" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="6" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="50"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="50" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="50" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="50" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="50" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="6" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="52" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="50" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="6" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="52" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="50" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="50" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="50" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="50" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="50" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="50" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="50" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="50" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="50" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="50" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="50" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="50" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="50" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="50" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="50" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="50" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="50" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="3" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="3" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="4" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="4" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="4" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="4" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="4" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="5" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="50" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="50" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="50" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="10" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="5" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="50" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="9" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="15" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="50" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="50" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="50" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="50" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="50" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="50" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="50" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="50" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="50" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="50" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="50" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="53" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="50" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="50" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="53" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="50" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="50" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="50" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="50" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="53" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="50" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="50" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="53" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="50" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="50" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="50" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="50" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="50" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="50" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="50" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="50" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="50" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="50" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="50" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="9" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="50" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="50" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="50" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="50" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="50" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="50" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" xfId="50" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="50" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="50" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="50" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="50" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="15" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="50" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="50" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="50" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="50" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="50" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="53" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="50" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="50" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="53" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="50" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="50" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="53" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="53" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="50" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="50" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="50" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="50" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="50" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" xfId="50" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="50" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="50" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="50" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="50" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="50" applyAlignment="1" quotePrefix="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="50" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -18470,7 +18453,7 @@
         <f t="shared" si="9"/>
         <v>304</v>
       </c>
-      <c r="H306" s="73" t="s">
+      <c r="H306" s="133" t="s">
         <v>14</v>
       </c>
       <c r="I306" s="112" t="s">
@@ -18927,7 +18910,7 @@
       <c r="H320" s="79" t="s">
         <v>14</v>
       </c>
-      <c r="I320" s="133" t="s">
+      <c r="I320" s="134" t="s">
         <v>720</v>
       </c>
       <c r="J320" s="81" t="s">
@@ -19123,7 +19106,7 @@
       <c r="H326" s="79" t="s">
         <v>14</v>
       </c>
-      <c r="I326" s="134" t="s">
+      <c r="I326" s="135" t="s">
         <v>735</v>
       </c>
       <c r="J326" s="120"/>
@@ -19168,7 +19151,7 @@
       <c r="A328" s="105" t="s">
         <v>739</v>
       </c>
-      <c r="B328" s="135" t="s">
+      <c r="B328" s="136" t="s">
         <v>25</v>
       </c>
       <c r="C328" s="107">
@@ -19218,7 +19201,7 @@
         <f t="shared" si="9"/>
         <v>327</v>
       </c>
-      <c r="H329" s="136" t="s">
+      <c r="H329" s="133" t="s">
         <v>14</v>
       </c>
       <c r="I329" s="87" t="s">
@@ -19562,7 +19545,7 @@
       <c r="A340" s="138" t="s">
         <v>768</v>
       </c>
-      <c r="B340" s="135" t="s">
+      <c r="B340" s="136" t="s">
         <v>63</v>
       </c>
       <c r="C340" s="76">
@@ -20212,7 +20195,7 @@
       <c r="A360" s="138" t="s">
         <v>810</v>
       </c>
-      <c r="B360" s="135" t="s">
+      <c r="B360" s="136" t="s">
         <v>63</v>
       </c>
       <c r="C360" s="76">
@@ -20264,7 +20247,7 @@
         <f t="shared" si="11"/>
         <v>359</v>
       </c>
-      <c r="H361" s="136" t="s">
+      <c r="H361" s="133" t="s">
         <v>14</v>
       </c>
       <c r="I361" s="87" t="s">
@@ -20618,7 +20601,7 @@
       <c r="A369" s="138" t="s">
         <v>833</v>
       </c>
-      <c r="B369" s="135" t="s">
+      <c r="B369" s="136" t="s">
         <v>834</v>
       </c>
       <c r="C369" s="76">
@@ -22600,7 +22583,7 @@
         <f t="shared" si="13"/>
         <v>425</v>
       </c>
-      <c r="H427" s="73" t="s">
+      <c r="H427" s="133" t="s">
         <v>14</v>
       </c>
       <c r="I427" s="21" t="s">
@@ -22631,7 +22614,7 @@
         <f t="shared" si="13"/>
         <v>426</v>
       </c>
-      <c r="H428" s="136" t="s">
+      <c r="H428" s="133" t="s">
         <v>14</v>
       </c>
       <c r="I428" s="112" t="s">
@@ -22801,7 +22784,7 @@
       <c r="H433" s="73" t="s">
         <v>14</v>
       </c>
-      <c r="I433" s="32" t="s">
+      <c r="I433" s="31" t="s">
         <v>978</v>
       </c>
       <c r="J433" s="64"/>
@@ -23368,7 +23351,7 @@
       <c r="C4" s="4" t="s">
         <v>984</v>
       </c>
-      <c r="E4" s="24" t="s">
+      <c r="E4" s="5" t="s">
         <v>985</v>
       </c>
     </row>
@@ -23389,7 +23372,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="25" t="s">
+      <c r="A7" s="24" t="s">
         <v>987</v>
       </c>
       <c r="B7" s="7" t="s">
@@ -23397,7 +23380,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="25" t="s">
+      <c r="A8" s="24" t="s">
         <v>989</v>
       </c>
       <c r="B8" s="7" t="s">
@@ -23405,7 +23388,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="25" t="s">
+      <c r="A9" s="24" t="s">
         <v>991</v>
       </c>
       <c r="B9" s="7" t="s">
@@ -23413,7 +23396,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="25" t="s">
+      <c r="A10" s="24" t="s">
         <v>993</v>
       </c>
       <c r="B10" s="7" t="s">
@@ -23421,7 +23404,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="24" t="s">
         <v>995</v>
       </c>
       <c r="B11" s="7" t="s">
@@ -23429,7 +23412,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="25" t="s">
+      <c r="A12" s="24" t="s">
         <v>997</v>
       </c>
       <c r="B12" s="7" t="s">
@@ -23437,7 +23420,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="25" t="s">
+      <c r="A13" s="24" t="s">
         <v>999</v>
       </c>
       <c r="B13" s="7" t="s">
@@ -23445,7 +23428,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="25" t="s">
+      <c r="A14" s="24" t="s">
         <v>1001</v>
       </c>
       <c r="B14" s="7" t="s">
@@ -23453,7 +23436,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="25" t="s">
+      <c r="A15" s="24" t="s">
         <v>1003</v>
       </c>
       <c r="B15" s="7" t="s">
@@ -23461,7 +23444,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="25" t="s">
+      <c r="A16" s="24" t="s">
         <v>1005</v>
       </c>
       <c r="B16" s="7" t="s">
@@ -23469,7 +23452,7 @@
       </c>
     </row>
     <row r="17" spans="1:3">
-      <c r="A17" s="25" t="s">
+      <c r="A17" s="24" t="s">
         <v>1007</v>
       </c>
       <c r="B17" s="7" t="s">
@@ -23477,7 +23460,7 @@
       </c>
     </row>
     <row r="18" spans="1:3">
-      <c r="A18" s="25" t="s">
+      <c r="A18" s="24" t="s">
         <v>1009</v>
       </c>
       <c r="B18" s="7" t="s">
@@ -23485,7 +23468,7 @@
       </c>
     </row>
     <row r="19" spans="1:3">
-      <c r="A19" s="25" t="s">
+      <c r="A19" s="24" t="s">
         <v>1011</v>
       </c>
       <c r="B19" s="7" t="s">
@@ -23493,7 +23476,7 @@
       </c>
     </row>
     <row r="20" spans="1:3">
-      <c r="A20" s="25" t="s">
+      <c r="A20" s="24" t="s">
         <v>1013</v>
       </c>
       <c r="B20" s="7" t="s">
@@ -23501,7 +23484,7 @@
       </c>
     </row>
     <row r="21" spans="1:3">
-      <c r="A21" s="25" t="s">
+      <c r="A21" s="24" t="s">
         <v>1015</v>
       </c>
       <c r="B21" s="7" t="s">
@@ -23509,7 +23492,7 @@
       </c>
     </row>
     <row r="22" spans="1:3">
-      <c r="A22" s="25" t="s">
+      <c r="A22" s="24" t="s">
         <v>1017</v>
       </c>
       <c r="B22" s="7" t="s">
@@ -23517,7 +23500,7 @@
       </c>
     </row>
     <row r="23" spans="1:3">
-      <c r="A23" s="25" t="s">
+      <c r="A23" s="24" t="s">
         <v>1019</v>
       </c>
       <c r="B23" s="7" t="s">
@@ -23525,7 +23508,7 @@
       </c>
     </row>
     <row r="24" spans="1:3">
-      <c r="A24" s="25" t="s">
+      <c r="A24" s="24" t="s">
         <v>1021</v>
       </c>
       <c r="B24" s="7" t="s">
@@ -23533,7 +23516,7 @@
       </c>
     </row>
     <row r="25" spans="1:3">
-      <c r="A25" s="25" t="s">
+      <c r="A25" s="24" t="s">
         <v>1023</v>
       </c>
       <c r="B25" s="7" t="s">
@@ -23541,13 +23524,13 @@
       </c>
     </row>
     <row r="26" spans="1:3">
-      <c r="A26" s="25"/>
+      <c r="A26" s="24"/>
     </row>
     <row r="27" spans="1:3">
-      <c r="A27" s="26" t="s">
+      <c r="A27" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="B27" s="27"/>
+      <c r="B27" s="26"/>
       <c r="C27" s="8" t="s">
         <v>1025</v>
       </c>
@@ -23577,8 +23560,8 @@
       </c>
     </row>
     <row r="31" spans="1:3">
-      <c r="A31" s="28"/>
-      <c r="B31" s="29"/>
+      <c r="A31" s="27"/>
+      <c r="B31" s="28"/>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="6" t="s">
@@ -23638,31 +23621,31 @@
       </c>
     </row>
     <row r="40" spans="1:3">
-      <c r="A40" s="28">
-        <v>1</v>
-      </c>
-      <c r="B40" s="29" t="s">
+      <c r="A40" s="27">
+        <v>1</v>
+      </c>
+      <c r="B40" s="28" t="s">
         <v>1032</v>
       </c>
     </row>
     <row r="41" spans="1:3">
-      <c r="A41" s="28">
+      <c r="A41" s="27">
         <v>2</v>
       </c>
-      <c r="B41" s="29" t="s">
+      <c r="B41" s="28" t="s">
         <v>1033</v>
       </c>
     </row>
     <row r="42" spans="1:3">
-      <c r="A42" s="28">
+      <c r="A42" s="27">
         <v>3</v>
       </c>
-      <c r="B42" s="29" t="s">
+      <c r="B42" s="28" t="s">
         <v>1034</v>
       </c>
     </row>
     <row r="43" spans="1:3">
-      <c r="A43" s="30"/>
+      <c r="A43" s="29"/>
       <c r="B43" s="3"/>
     </row>
     <row r="44" spans="1:3">
@@ -23683,7 +23666,7 @@
       </c>
     </row>
     <row r="46" spans="1:3">
-      <c r="A46" s="30">
+      <c r="A46" s="29">
         <v>1</v>
       </c>
       <c r="B46" s="3" t="s">
@@ -23691,7 +23674,7 @@
       </c>
     </row>
     <row r="47" spans="1:3">
-      <c r="A47" s="30">
+      <c r="A47" s="29">
         <v>2</v>
       </c>
       <c r="B47" s="3" t="s">
@@ -23699,7 +23682,7 @@
       </c>
     </row>
     <row r="48" spans="1:3">
-      <c r="A48" s="30">
+      <c r="A48" s="29">
         <v>3</v>
       </c>
       <c r="B48" s="3" t="s">
@@ -23707,7 +23690,7 @@
       </c>
     </row>
     <row r="49" spans="1:3">
-      <c r="A49" s="30">
+      <c r="A49" s="29">
         <v>4</v>
       </c>
       <c r="B49" s="3" t="s">
@@ -23715,7 +23698,7 @@
       </c>
     </row>
     <row r="50" spans="1:3">
-      <c r="A50" s="30">
+      <c r="A50" s="29">
         <v>5</v>
       </c>
       <c r="B50" s="3" t="s">
@@ -23723,7 +23706,7 @@
       </c>
     </row>
     <row r="51" spans="1:3">
-      <c r="A51" s="30">
+      <c r="A51" s="29">
         <v>6</v>
       </c>
       <c r="B51" s="3" t="s">
@@ -23731,7 +23714,7 @@
       </c>
     </row>
     <row r="52" spans="1:3">
-      <c r="A52" s="30">
+      <c r="A52" s="29">
         <v>7</v>
       </c>
       <c r="B52" s="3" t="s">
@@ -23739,7 +23722,7 @@
       </c>
     </row>
     <row r="53" spans="1:3">
-      <c r="A53" s="30">
+      <c r="A53" s="29">
         <v>8</v>
       </c>
       <c r="B53" s="3" t="s">
@@ -23747,7 +23730,7 @@
       </c>
     </row>
     <row r="55" spans="1:3">
-      <c r="A55" s="26" t="s">
+      <c r="A55" s="25" t="s">
         <v>49</v>
       </c>
       <c r="C55" s="15" t="s">
@@ -23819,7 +23802,7 @@
       </c>
     </row>
     <row r="66" spans="1:3">
-      <c r="A66" s="26" t="s">
+      <c r="A66" s="25" t="s">
         <v>66</v>
       </c>
       <c r="C66" s="8" t="s">
@@ -23867,7 +23850,7 @@
       </c>
     </row>
     <row r="73" spans="1:3">
-      <c r="A73" s="26" t="s">
+      <c r="A73" s="25" t="s">
         <v>69</v>
       </c>
       <c r="C73" s="8" t="s">
@@ -23947,79 +23930,79 @@
       </c>
     </row>
     <row r="84" spans="1:3">
-      <c r="A84" s="31" t="s">
+      <c r="A84" s="30" t="s">
         <v>987</v>
       </c>
-      <c r="B84" s="32" t="s">
+      <c r="B84" s="31" t="s">
         <v>1055</v>
       </c>
     </row>
     <row r="85" spans="1:3">
-      <c r="A85" s="31" t="s">
+      <c r="A85" s="30" t="s">
         <v>989</v>
       </c>
-      <c r="B85" s="32" t="s">
+      <c r="B85" s="31" t="s">
         <v>1056</v>
       </c>
     </row>
     <row r="86" spans="1:3">
-      <c r="A86" s="31" t="s">
+      <c r="A86" s="30" t="s">
         <v>991</v>
       </c>
-      <c r="B86" s="32" t="s">
+      <c r="B86" s="31" t="s">
         <v>1057</v>
       </c>
     </row>
     <row r="87" spans="1:3">
-      <c r="A87" s="31" t="s">
+      <c r="A87" s="30" t="s">
         <v>993</v>
       </c>
-      <c r="B87" s="32" t="s">
+      <c r="B87" s="31" t="s">
         <v>1058</v>
       </c>
     </row>
     <row r="88" spans="1:3">
-      <c r="A88" s="31" t="s">
+      <c r="A88" s="30" t="s">
         <v>995</v>
       </c>
-      <c r="B88" s="32" t="s">
+      <c r="B88" s="31" t="s">
         <v>1059</v>
       </c>
     </row>
     <row r="89" spans="1:3">
-      <c r="A89" s="31" t="s">
+      <c r="A89" s="30" t="s">
         <v>997</v>
       </c>
-      <c r="B89" s="32" t="s">
+      <c r="B89" s="31" t="s">
         <v>1060</v>
       </c>
     </row>
     <row r="90" spans="1:3">
-      <c r="A90" s="31" t="s">
+      <c r="A90" s="30" t="s">
         <v>999</v>
       </c>
-      <c r="B90" s="32" t="s">
+      <c r="B90" s="31" t="s">
         <v>1061</v>
       </c>
     </row>
     <row r="91" spans="1:3">
-      <c r="A91" s="31" t="s">
+      <c r="A91" s="30" t="s">
         <v>1001</v>
       </c>
-      <c r="B91" s="32" t="s">
+      <c r="B91" s="31" t="s">
         <v>1062</v>
       </c>
     </row>
     <row r="92" spans="1:3">
-      <c r="A92" s="31" t="s">
+      <c r="A92" s="30" t="s">
         <v>1003</v>
       </c>
-      <c r="B92" s="32" t="s">
+      <c r="B92" s="31" t="s">
         <v>1063</v>
       </c>
     </row>
     <row r="93" spans="1:3">
-      <c r="A93" s="31">
+      <c r="A93" s="30">
         <v>99</v>
       </c>
       <c r="B93" s="7" t="s">
@@ -24223,7 +24206,7 @@
       </c>
     </row>
     <row r="122" spans="1:3">
-      <c r="A122" s="26" t="s">
+      <c r="A122" s="25" t="s">
         <v>99</v>
       </c>
       <c r="C122" s="8" t="s">
@@ -24239,7 +24222,7 @@
       </c>
     </row>
     <row r="124" spans="1:3">
-      <c r="A124" s="25" t="s">
+      <c r="A124" s="24" t="s">
         <v>987</v>
       </c>
       <c r="B124" s="7" t="s">
@@ -24247,7 +24230,7 @@
       </c>
     </row>
     <row r="125" spans="1:3">
-      <c r="A125" s="25" t="s">
+      <c r="A125" s="24" t="s">
         <v>989</v>
       </c>
       <c r="B125" s="7" t="s">
@@ -24255,7 +24238,7 @@
       </c>
     </row>
     <row r="126" spans="1:3">
-      <c r="A126" s="25" t="s">
+      <c r="A126" s="24" t="s">
         <v>991</v>
       </c>
       <c r="B126" s="7" t="s">
@@ -24263,7 +24246,7 @@
       </c>
     </row>
     <row r="127" spans="1:3">
-      <c r="A127" s="25" t="s">
+      <c r="A127" s="24" t="s">
         <v>993</v>
       </c>
       <c r="B127" s="7" t="s">
@@ -24271,7 +24254,7 @@
       </c>
     </row>
     <row r="128" spans="1:3">
-      <c r="A128" s="25" t="s">
+      <c r="A128" s="24" t="s">
         <v>995</v>
       </c>
       <c r="B128" s="7" t="s">
@@ -24279,7 +24262,7 @@
       </c>
     </row>
     <row r="129" spans="1:3">
-      <c r="A129" s="25" t="s">
+      <c r="A129" s="24" t="s">
         <v>997</v>
       </c>
       <c r="B129" s="7" t="s">
@@ -24287,7 +24270,7 @@
       </c>
     </row>
     <row r="130" spans="1:3">
-      <c r="A130" s="25" t="s">
+      <c r="A130" s="24" t="s">
         <v>999</v>
       </c>
       <c r="B130" s="7" t="s">
@@ -24295,7 +24278,7 @@
       </c>
     </row>
     <row r="131" spans="1:3">
-      <c r="A131" s="25" t="s">
+      <c r="A131" s="24" t="s">
         <v>1001</v>
       </c>
       <c r="B131" s="7" t="s">
@@ -24303,7 +24286,7 @@
       </c>
     </row>
     <row r="132" spans="1:3">
-      <c r="A132" s="25" t="s">
+      <c r="A132" s="24" t="s">
         <v>1003</v>
       </c>
       <c r="B132" s="7" t="s">
@@ -24463,42 +24446,42 @@
       </c>
     </row>
     <row r="155" spans="1:3">
-      <c r="A155" s="33">
-        <v>1</v>
-      </c>
-      <c r="B155" s="32" t="s">
+      <c r="A155" s="32">
+        <v>1</v>
+      </c>
+      <c r="B155" s="31" t="s">
         <v>1030</v>
       </c>
     </row>
     <row r="156" spans="1:3">
-      <c r="A156" s="33">
+      <c r="A156" s="32">
         <v>2</v>
       </c>
-      <c r="B156" s="32" t="s">
+      <c r="B156" s="31" t="s">
         <v>1085</v>
       </c>
     </row>
     <row r="157" spans="1:3">
-      <c r="A157" s="33">
+      <c r="A157" s="32">
         <v>3</v>
       </c>
-      <c r="B157" s="32" t="s">
+      <c r="B157" s="31" t="s">
         <v>1086</v>
       </c>
     </row>
     <row r="158" spans="1:3">
-      <c r="A158" s="33">
+      <c r="A158" s="32">
         <v>4</v>
       </c>
-      <c r="B158" s="32" t="s">
+      <c r="B158" s="31" t="s">
         <v>1087</v>
       </c>
     </row>
     <row r="159" spans="1:3">
-      <c r="A159" s="33">
+      <c r="A159" s="32">
         <v>5</v>
       </c>
-      <c r="B159" s="32" t="s">
+      <c r="B159" s="31" t="s">
         <v>1088</v>
       </c>
     </row>
@@ -24515,7 +24498,7 @@
       <c r="B161" s="12"/>
     </row>
     <row r="162" spans="1:3">
-      <c r="A162" s="26" t="s">
+      <c r="A162" s="25" t="s">
         <v>111</v>
       </c>
       <c r="C162" s="8" t="s">
@@ -24571,7 +24554,7 @@
       </c>
     </row>
     <row r="170" spans="1:3">
-      <c r="A170" s="25" t="s">
+      <c r="A170" s="24" t="s">
         <v>987</v>
       </c>
       <c r="B170" s="7" t="s">
@@ -24579,7 +24562,7 @@
       </c>
     </row>
     <row r="171" spans="1:3">
-      <c r="A171" s="25" t="s">
+      <c r="A171" s="24" t="s">
         <v>989</v>
       </c>
       <c r="B171" s="7" t="s">
@@ -24587,7 +24570,7 @@
       </c>
     </row>
     <row r="172" spans="1:3">
-      <c r="A172" s="25" t="s">
+      <c r="A172" s="24" t="s">
         <v>991</v>
       </c>
       <c r="B172" s="7" t="s">
@@ -24595,7 +24578,7 @@
       </c>
     </row>
     <row r="173" spans="1:3">
-      <c r="A173" s="25" t="s">
+      <c r="A173" s="24" t="s">
         <v>993</v>
       </c>
       <c r="B173" s="7" t="s">
@@ -24603,7 +24586,7 @@
       </c>
     </row>
     <row r="174" spans="1:3">
-      <c r="A174" s="25" t="s">
+      <c r="A174" s="24" t="s">
         <v>995</v>
       </c>
       <c r="B174" s="7" t="s">
@@ -24611,7 +24594,7 @@
       </c>
     </row>
     <row r="175" spans="1:3">
-      <c r="A175" s="25" t="s">
+      <c r="A175" s="24" t="s">
         <v>997</v>
       </c>
       <c r="B175" s="7" t="s">
@@ -24619,7 +24602,7 @@
       </c>
     </row>
     <row r="176" spans="1:3">
-      <c r="A176" s="25" t="s">
+      <c r="A176" s="24" t="s">
         <v>999</v>
       </c>
       <c r="B176" s="7" t="s">
@@ -24627,7 +24610,7 @@
       </c>
     </row>
     <row r="177" spans="1:3">
-      <c r="A177" s="25" t="s">
+      <c r="A177" s="24" t="s">
         <v>1001</v>
       </c>
       <c r="B177" s="7" t="s">
@@ -25305,7 +25288,7 @@
       <c r="A275" s="6" t="s">
         <v>416</v>
       </c>
-      <c r="C275" s="34" t="s">
+      <c r="C275" s="33" t="s">
         <v>415</v>
       </c>
     </row>
@@ -25377,7 +25360,7 @@
       <c r="A285" s="6" t="s">
         <v>419</v>
       </c>
-      <c r="C285" s="34" t="s">
+      <c r="C285" s="33" t="s">
         <v>418</v>
       </c>
     </row>
@@ -25601,7 +25584,7 @@
       </c>
     </row>
     <row r="317" spans="1:3">
-      <c r="A317" s="25" t="s">
+      <c r="A317" s="24" t="s">
         <v>987</v>
       </c>
       <c r="B317" s="7" t="s">
@@ -25609,7 +25592,7 @@
       </c>
     </row>
     <row r="318" spans="1:3">
-      <c r="A318" s="25" t="s">
+      <c r="A318" s="24" t="s">
         <v>989</v>
       </c>
       <c r="B318" s="7" t="s">
@@ -25617,7 +25600,7 @@
       </c>
     </row>
     <row r="319" spans="1:3">
-      <c r="A319" s="25" t="s">
+      <c r="A319" s="24" t="s">
         <v>991</v>
       </c>
       <c r="B319" s="7" t="s">
@@ -25625,7 +25608,7 @@
       </c>
     </row>
     <row r="320" spans="1:3">
-      <c r="A320" s="25" t="s">
+      <c r="A320" s="24" t="s">
         <v>993</v>
       </c>
       <c r="B320" s="7" t="s">
@@ -25633,7 +25616,7 @@
       </c>
     </row>
     <row r="321" spans="1:3">
-      <c r="A321" s="25" t="s">
+      <c r="A321" s="24" t="s">
         <v>995</v>
       </c>
       <c r="B321" s="7" t="s">
@@ -25641,7 +25624,7 @@
       </c>
     </row>
     <row r="322" spans="1:3">
-      <c r="A322" s="25" t="s">
+      <c r="A322" s="24" t="s">
         <v>997</v>
       </c>
       <c r="B322" s="7" t="s">
@@ -25649,7 +25632,7 @@
       </c>
     </row>
     <row r="323" spans="1:3">
-      <c r="A323" s="25" t="s">
+      <c r="A323" s="24" t="s">
         <v>999</v>
       </c>
       <c r="B323" s="7" t="s">
@@ -25657,7 +25640,7 @@
       </c>
     </row>
     <row r="324" spans="1:3">
-      <c r="A324" s="25" t="s">
+      <c r="A324" s="24" t="s">
         <v>1001</v>
       </c>
       <c r="B324" s="7" t="s">
@@ -25665,7 +25648,7 @@
       </c>
     </row>
     <row r="325" spans="1:3">
-      <c r="A325" s="25" t="s">
+      <c r="A325" s="24" t="s">
         <v>1003</v>
       </c>
       <c r="B325" s="7" t="s">
@@ -25786,7 +25769,7 @@
       </c>
     </row>
     <row r="342" spans="1:3">
-      <c r="A342" s="30">
+      <c r="A342" s="29">
         <v>1</v>
       </c>
       <c r="B342" s="3" t="s">
@@ -25794,7 +25777,7 @@
       </c>
     </row>
     <row r="343" spans="1:3">
-      <c r="A343" s="30">
+      <c r="A343" s="29">
         <v>2</v>
       </c>
       <c r="B343" s="3" t="s">
@@ -25802,7 +25785,7 @@
       </c>
     </row>
     <row r="344" spans="1:3">
-      <c r="A344" s="30">
+      <c r="A344" s="29">
         <v>3</v>
       </c>
       <c r="B344" s="3" t="s">
@@ -25810,7 +25793,7 @@
       </c>
     </row>
     <row r="345" spans="1:3">
-      <c r="A345" s="30">
+      <c r="A345" s="29">
         <v>4</v>
       </c>
       <c r="B345" s="3" t="s">
@@ -25842,7 +25825,7 @@
       </c>
     </row>
     <row r="350" spans="1:3">
-      <c r="A350" s="30">
+      <c r="A350" s="29">
         <v>1</v>
       </c>
       <c r="B350" s="3" t="s">
@@ -25850,7 +25833,7 @@
       </c>
     </row>
     <row r="351" spans="1:3">
-      <c r="A351" s="30">
+      <c r="A351" s="29">
         <v>2</v>
       </c>
       <c r="B351" s="3" t="s">
@@ -25858,7 +25841,7 @@
       </c>
     </row>
     <row r="352" spans="1:3">
-      <c r="A352" s="30">
+      <c r="A352" s="29">
         <v>3</v>
       </c>
       <c r="B352" s="3" t="s">
@@ -25866,7 +25849,7 @@
       </c>
     </row>
     <row r="353" spans="1:3">
-      <c r="A353" s="30">
+      <c r="A353" s="29">
         <v>4</v>
       </c>
       <c r="B353" s="3" t="s">
@@ -25874,7 +25857,7 @@
       </c>
     </row>
     <row r="354" spans="1:3">
-      <c r="A354" s="30">
+      <c r="A354" s="29">
         <v>5</v>
       </c>
       <c r="B354" s="3" t="s">
@@ -25915,7 +25898,7 @@
       </c>
     </row>
     <row r="360" spans="1:3">
-      <c r="A360" s="35">
+      <c r="A360" s="34">
         <v>3</v>
       </c>
       <c r="B360" s="11" t="s">
@@ -25923,7 +25906,7 @@
       </c>
     </row>
     <row r="361" spans="1:3">
-      <c r="A361" s="35">
+      <c r="A361" s="34">
         <v>4</v>
       </c>
       <c r="B361" s="11" t="s">
@@ -25956,7 +25939,7 @@
       </c>
     </row>
     <row r="366" spans="1:3">
-      <c r="A366" s="30">
+      <c r="A366" s="29">
         <v>1</v>
       </c>
       <c r="B366" s="3" t="s">
@@ -25964,7 +25947,7 @@
       </c>
     </row>
     <row r="367" spans="1:3">
-      <c r="A367" s="30">
+      <c r="A367" s="29">
         <v>2</v>
       </c>
       <c r="B367" s="3" t="s">
@@ -25972,7 +25955,7 @@
       </c>
     </row>
     <row r="368" spans="1:3">
-      <c r="A368" s="30">
+      <c r="A368" s="29">
         <v>3</v>
       </c>
       <c r="B368" s="3" t="s">
@@ -25980,7 +25963,7 @@
       </c>
     </row>
     <row r="369" spans="1:3">
-      <c r="A369" s="30">
+      <c r="A369" s="29">
         <v>4</v>
       </c>
       <c r="B369" s="3" t="s">
@@ -25988,7 +25971,7 @@
       </c>
     </row>
     <row r="370" spans="1:3">
-      <c r="A370" s="30">
+      <c r="A370" s="29">
         <v>5</v>
       </c>
       <c r="B370" s="3" t="s">
@@ -26020,7 +26003,7 @@
       </c>
     </row>
     <row r="375" spans="1:3">
-      <c r="A375" s="30">
+      <c r="A375" s="29">
         <v>1</v>
       </c>
       <c r="B375" s="3" t="s">
@@ -26028,7 +26011,7 @@
       </c>
     </row>
     <row r="376" spans="1:3">
-      <c r="A376" s="30">
+      <c r="A376" s="29">
         <v>2</v>
       </c>
       <c r="B376" s="3" t="s">
@@ -26036,7 +26019,7 @@
       </c>
     </row>
     <row r="377" spans="1:3">
-      <c r="A377" s="30">
+      <c r="A377" s="29">
         <v>3</v>
       </c>
       <c r="B377" s="3" t="s">
@@ -26044,7 +26027,7 @@
       </c>
     </row>
     <row r="378" spans="1:3">
-      <c r="A378" s="30">
+      <c r="A378" s="29">
         <v>4</v>
       </c>
       <c r="B378" s="3" t="s">
@@ -26052,7 +26035,7 @@
       </c>
     </row>
     <row r="379" spans="1:3">
-      <c r="A379" s="30">
+      <c r="A379" s="29">
         <v>5</v>
       </c>
       <c r="B379" s="3" t="s">
@@ -26085,7 +26068,7 @@
       </c>
     </row>
     <row r="384" spans="1:3">
-      <c r="A384" s="30">
+      <c r="A384" s="29">
         <v>1</v>
       </c>
       <c r="B384" s="3" t="s">
@@ -26093,7 +26076,7 @@
       </c>
     </row>
     <row r="385" spans="1:3">
-      <c r="A385" s="30">
+      <c r="A385" s="29">
         <v>2</v>
       </c>
       <c r="B385" s="3" t="s">
@@ -26101,7 +26084,7 @@
       </c>
     </row>
     <row r="386" spans="1:3">
-      <c r="A386" s="30">
+      <c r="A386" s="29">
         <v>3</v>
       </c>
       <c r="B386" s="3" t="s">
@@ -26109,7 +26092,7 @@
       </c>
     </row>
     <row r="387" spans="1:3">
-      <c r="A387" s="30">
+      <c r="A387" s="29">
         <v>4</v>
       </c>
       <c r="B387" s="3" t="s">
@@ -26117,7 +26100,7 @@
       </c>
     </row>
     <row r="388" spans="1:3">
-      <c r="A388" s="30">
+      <c r="A388" s="29">
         <v>5</v>
       </c>
       <c r="B388" s="3" t="s">
@@ -26125,7 +26108,7 @@
       </c>
     </row>
     <row r="389" spans="1:3">
-      <c r="A389" s="35">
+      <c r="A389" s="34">
         <v>6</v>
       </c>
       <c r="B389" s="11" t="s">
@@ -26158,7 +26141,7 @@
       </c>
     </row>
     <row r="394" spans="1:3">
-      <c r="A394" s="30">
+      <c r="A394" s="29">
         <v>1</v>
       </c>
       <c r="B394" s="3" t="s">
@@ -26166,15 +26149,15 @@
       </c>
     </row>
     <row r="395" spans="1:3">
-      <c r="A395" s="30">
+      <c r="A395" s="29">
         <v>2</v>
       </c>
-      <c r="B395" s="36" t="s">
+      <c r="B395" s="35" t="s">
         <v>1185</v>
       </c>
     </row>
     <row r="396" spans="1:3">
-      <c r="A396" s="30">
+      <c r="A396" s="29">
         <v>3</v>
       </c>
       <c r="B396" s="3" t="s">
@@ -26182,7 +26165,7 @@
       </c>
     </row>
     <row r="397" spans="1:3">
-      <c r="A397" s="30">
+      <c r="A397" s="29">
         <v>4</v>
       </c>
       <c r="B397" s="3" t="s">
@@ -26190,7 +26173,7 @@
       </c>
     </row>
     <row r="398" spans="1:3">
-      <c r="A398" s="30">
+      <c r="A398" s="29">
         <v>5</v>
       </c>
       <c r="B398" s="3" t="s">
@@ -26223,7 +26206,7 @@
       </c>
     </row>
     <row r="403" spans="1:3">
-      <c r="A403" s="30">
+      <c r="A403" s="29">
         <v>1</v>
       </c>
       <c r="B403" s="3" t="s">
@@ -26231,7 +26214,7 @@
       </c>
     </row>
     <row r="404" spans="1:3">
-      <c r="A404" s="30">
+      <c r="A404" s="29">
         <v>2</v>
       </c>
       <c r="B404" s="3" t="s">
@@ -26239,7 +26222,7 @@
       </c>
     </row>
     <row r="405" spans="1:3">
-      <c r="A405" s="30">
+      <c r="A405" s="29">
         <v>3</v>
       </c>
       <c r="B405" s="3" t="s">
@@ -26247,7 +26230,7 @@
       </c>
     </row>
     <row r="406" spans="1:3">
-      <c r="A406" s="30">
+      <c r="A406" s="29">
         <v>4</v>
       </c>
       <c r="B406" s="3" t="s">
@@ -26279,7 +26262,7 @@
       </c>
     </row>
     <row r="411" spans="1:3">
-      <c r="A411" s="30">
+      <c r="A411" s="29">
         <v>1</v>
       </c>
       <c r="B411" s="3" t="s">
@@ -26287,7 +26270,7 @@
       </c>
     </row>
     <row r="412" spans="1:3">
-      <c r="A412" s="30">
+      <c r="A412" s="29">
         <v>2</v>
       </c>
       <c r="B412" s="3" t="s">
@@ -26295,7 +26278,7 @@
       </c>
     </row>
     <row r="413" spans="1:3">
-      <c r="A413" s="30">
+      <c r="A413" s="29">
         <v>3</v>
       </c>
       <c r="B413" s="3" t="s">
@@ -26303,7 +26286,7 @@
       </c>
     </row>
     <row r="414" spans="1:3">
-      <c r="A414" s="30">
+      <c r="A414" s="29">
         <v>4</v>
       </c>
       <c r="B414" s="3" t="s">
@@ -26336,7 +26319,7 @@
       </c>
     </row>
     <row r="419" spans="1:3">
-      <c r="A419" s="30">
+      <c r="A419" s="29">
         <v>1</v>
       </c>
       <c r="B419" s="3" t="s">
@@ -26376,15 +26359,15 @@
       </c>
     </row>
     <row r="424" spans="1:3">
-      <c r="A424" s="30"/>
+      <c r="A424" s="29"/>
       <c r="B424" s="3"/>
     </row>
     <row r="425" spans="1:3">
-      <c r="A425" s="26"/>
-      <c r="B425" s="26"/>
+      <c r="A425" s="25"/>
+      <c r="B425" s="25"/>
     </row>
     <row r="426" spans="1:3">
-      <c r="A426" s="26" t="s">
+      <c r="A426" s="25" t="s">
         <v>722</v>
       </c>
       <c r="B426" s="3"/>
@@ -26433,10 +26416,10 @@
       </c>
     </row>
     <row r="432" spans="1:3">
-      <c r="A432" s="37"/>
+      <c r="A432" s="36"/>
     </row>
     <row r="433" spans="1:3">
-      <c r="A433" s="26" t="s">
+      <c r="A433" s="25" t="s">
         <v>728</v>
       </c>
       <c r="B433" s="3"/>
@@ -26506,7 +26489,7 @@
       </c>
     </row>
     <row r="442" spans="1:3">
-      <c r="A442" s="30">
+      <c r="A442" s="29">
         <v>1</v>
       </c>
       <c r="B442" s="3" t="s">
@@ -26514,7 +26497,7 @@
       </c>
     </row>
     <row r="443" spans="1:3">
-      <c r="A443" s="30">
+      <c r="A443" s="29">
         <v>2</v>
       </c>
       <c r="B443" s="3" t="s">
@@ -26522,7 +26505,7 @@
       </c>
     </row>
     <row r="444" spans="1:3">
-      <c r="A444" s="30">
+      <c r="A444" s="29">
         <v>3</v>
       </c>
       <c r="B444" s="3" t="s">
@@ -26530,7 +26513,7 @@
       </c>
     </row>
     <row r="445" spans="1:3">
-      <c r="A445" s="30">
+      <c r="A445" s="29">
         <v>4</v>
       </c>
       <c r="B445" s="3" t="s">
@@ -26538,7 +26521,7 @@
       </c>
     </row>
     <row r="446" spans="1:3">
-      <c r="A446" s="30">
+      <c r="A446" s="29">
         <v>5</v>
       </c>
       <c r="B446" s="3" t="s">
@@ -26691,50 +26674,50 @@
       </c>
     </row>
     <row r="468" spans="1:3">
-      <c r="A468" s="35">
-        <v>1</v>
-      </c>
-      <c r="B468" s="35" t="s">
+      <c r="A468" s="34">
+        <v>1</v>
+      </c>
+      <c r="B468" s="34" t="s">
         <v>1214</v>
       </c>
     </row>
     <row r="469" spans="1:3">
-      <c r="A469" s="35">
+      <c r="A469" s="34">
         <v>2</v>
       </c>
-      <c r="B469" s="35" t="s">
+      <c r="B469" s="34" t="s">
         <v>1215</v>
       </c>
     </row>
     <row r="470" spans="1:3">
-      <c r="A470" s="35">
+      <c r="A470" s="34">
         <v>3</v>
       </c>
-      <c r="B470" s="35" t="s">
+      <c r="B470" s="34" t="s">
         <v>1216</v>
       </c>
     </row>
     <row r="471" spans="1:3">
-      <c r="A471" s="35">
+      <c r="A471" s="34">
         <v>4</v>
       </c>
-      <c r="B471" s="35" t="s">
+      <c r="B471" s="34" t="s">
         <v>1217</v>
       </c>
     </row>
     <row r="472" spans="1:3">
-      <c r="A472" s="35">
+      <c r="A472" s="34">
         <v>5</v>
       </c>
-      <c r="B472" s="35" t="s">
+      <c r="B472" s="34" t="s">
         <v>1218</v>
       </c>
     </row>
     <row r="473" spans="1:3">
-      <c r="A473" s="35">
+      <c r="A473" s="34">
         <v>6</v>
       </c>
-      <c r="B473" s="35" t="s">
+      <c r="B473" s="34" t="s">
         <v>1141</v>
       </c>
     </row>
@@ -26747,8 +26730,8 @@
       </c>
     </row>
     <row r="475" spans="1:3">
-      <c r="A475" s="38"/>
-      <c r="B475" s="39"/>
+      <c r="A475" s="37"/>
+      <c r="B475" s="38"/>
     </row>
     <row r="476" spans="1:3">
       <c r="A476" s="6" t="s">
@@ -26807,7 +26790,7 @@
       </c>
     </row>
     <row r="484" spans="1:3">
-      <c r="A484" s="26" t="s">
+      <c r="A484" s="25" t="s">
         <v>825</v>
       </c>
       <c r="C484" s="8" t="s">
@@ -26867,7 +26850,7 @@
       <c r="B491" s="12"/>
     </row>
     <row r="492" spans="1:3">
-      <c r="A492" s="26" t="s">
+      <c r="A492" s="25" t="s">
         <v>828</v>
       </c>
       <c r="C492" s="8" t="s">
@@ -26919,7 +26902,7 @@
       <c r="B498" s="12"/>
     </row>
     <row r="499" spans="1:3">
-      <c r="A499" s="26" t="s">
+      <c r="A499" s="25" t="s">
         <v>831</v>
       </c>
       <c r="C499" s="8" t="s">
@@ -26971,7 +26954,7 @@
       <c r="B505" s="12"/>
     </row>
     <row r="506" spans="1:3">
-      <c r="A506" s="26" t="s">
+      <c r="A506" s="25" t="s">
         <v>834</v>
       </c>
       <c r="C506" s="8" t="s">
@@ -27027,7 +27010,7 @@
       </c>
     </row>
     <row r="514" spans="1:3">
-      <c r="A514" s="25" t="s">
+      <c r="A514" s="24" t="s">
         <v>987</v>
       </c>
       <c r="B514" s="12" t="s">
@@ -27035,7 +27018,7 @@
       </c>
     </row>
     <row r="515" spans="1:3">
-      <c r="A515" s="25" t="s">
+      <c r="A515" s="24" t="s">
         <v>989</v>
       </c>
       <c r="B515" s="12" t="s">
@@ -27043,7 +27026,7 @@
       </c>
     </row>
     <row r="516" spans="1:3">
-      <c r="A516" s="25" t="s">
+      <c r="A516" s="24" t="s">
         <v>991</v>
       </c>
       <c r="B516" s="12" t="s">
@@ -27051,7 +27034,7 @@
       </c>
     </row>
     <row r="517" spans="1:3">
-      <c r="A517" s="25" t="s">
+      <c r="A517" s="24" t="s">
         <v>993</v>
       </c>
       <c r="B517" s="12" t="s">
@@ -27059,7 +27042,7 @@
       </c>
     </row>
     <row r="518" spans="1:3">
-      <c r="A518" s="25" t="s">
+      <c r="A518" s="24" t="s">
         <v>995</v>
       </c>
       <c r="B518" s="12" t="s">
@@ -27067,7 +27050,7 @@
       </c>
     </row>
     <row r="519" spans="1:3">
-      <c r="A519" s="25" t="s">
+      <c r="A519" s="24" t="s">
         <v>997</v>
       </c>
       <c r="B519" s="12" t="s">
@@ -27075,7 +27058,7 @@
       </c>
     </row>
     <row r="520" spans="1:3">
-      <c r="A520" s="25" t="s">
+      <c r="A520" s="24" t="s">
         <v>999</v>
       </c>
       <c r="B520" s="12" t="s">
@@ -27083,7 +27066,7 @@
       </c>
     </row>
     <row r="521" spans="1:3">
-      <c r="A521" s="25" t="s">
+      <c r="A521" s="24" t="s">
         <v>1001</v>
       </c>
       <c r="B521" s="12" t="s">
@@ -27091,7 +27074,7 @@
       </c>
     </row>
     <row r="522" spans="1:3">
-      <c r="A522" s="25" t="s">
+      <c r="A522" s="24" t="s">
         <v>1003</v>
       </c>
       <c r="B522" s="12" t="s">
@@ -27123,7 +27106,7 @@
       </c>
     </row>
     <row r="527" spans="1:3">
-      <c r="A527" s="25" t="s">
+      <c r="A527" s="24" t="s">
         <v>987</v>
       </c>
       <c r="B527" s="12" t="s">
@@ -27131,7 +27114,7 @@
       </c>
     </row>
     <row r="528" spans="1:3">
-      <c r="A528" s="25" t="s">
+      <c r="A528" s="24" t="s">
         <v>989</v>
       </c>
       <c r="B528" s="12" t="s">
@@ -27139,7 +27122,7 @@
       </c>
     </row>
     <row r="529" spans="1:3">
-      <c r="A529" s="25" t="s">
+      <c r="A529" s="24" t="s">
         <v>991</v>
       </c>
       <c r="B529" s="12" t="s">
@@ -27147,7 +27130,7 @@
       </c>
     </row>
     <row r="530" spans="1:3">
-      <c r="A530" s="25" t="s">
+      <c r="A530" s="24" t="s">
         <v>993</v>
       </c>
       <c r="B530" s="12" t="s">
@@ -27155,7 +27138,7 @@
       </c>
     </row>
     <row r="531" spans="1:3">
-      <c r="A531" s="25" t="s">
+      <c r="A531" s="24" t="s">
         <v>995</v>
       </c>
       <c r="B531" s="12" t="s">
@@ -27163,7 +27146,7 @@
       </c>
     </row>
     <row r="532" spans="1:3">
-      <c r="A532" s="25" t="s">
+      <c r="A532" s="24" t="s">
         <v>997</v>
       </c>
       <c r="B532" s="12" t="s">
@@ -27171,7 +27154,7 @@
       </c>
     </row>
     <row r="533" spans="1:3">
-      <c r="A533" s="25" t="s">
+      <c r="A533" s="24" t="s">
         <v>999</v>
       </c>
       <c r="B533" s="7" t="s">
@@ -27179,7 +27162,7 @@
       </c>
     </row>
     <row r="534" spans="1:3">
-      <c r="A534" s="25" t="s">
+      <c r="A534" s="24" t="s">
         <v>1001</v>
       </c>
       <c r="B534" s="7" t="s">
@@ -27187,7 +27170,7 @@
       </c>
     </row>
     <row r="535" spans="1:3">
-      <c r="A535" s="25" t="s">
+      <c r="A535" s="24" t="s">
         <v>1003</v>
       </c>
       <c r="B535" s="7" t="s">
@@ -27220,34 +27203,34 @@
       </c>
     </row>
     <row r="540" spans="1:3">
-      <c r="A540" s="35">
-        <v>1</v>
-      </c>
-      <c r="B540" s="35" t="s">
+      <c r="A540" s="34">
+        <v>1</v>
+      </c>
+      <c r="B540" s="34" t="s">
         <v>1247</v>
       </c>
     </row>
     <row r="541" spans="1:3">
-      <c r="A541" s="35">
+      <c r="A541" s="34">
         <v>2</v>
       </c>
-      <c r="B541" s="35" t="s">
+      <c r="B541" s="34" t="s">
         <v>1248</v>
       </c>
     </row>
     <row r="542" spans="1:3">
-      <c r="A542" s="35">
+      <c r="A542" s="34">
         <v>3</v>
       </c>
-      <c r="B542" s="35" t="s">
+      <c r="B542" s="34" t="s">
         <v>1249</v>
       </c>
     </row>
     <row r="543" spans="1:3">
-      <c r="A543" s="35">
+      <c r="A543" s="34">
         <v>4</v>
       </c>
-      <c r="B543" s="35" t="s">
+      <c r="B543" s="34" t="s">
         <v>1250</v>
       </c>
     </row>
@@ -27260,7 +27243,7 @@
       </c>
     </row>
     <row r="545" spans="1:3">
-      <c r="A545" s="30"/>
+      <c r="A545" s="29"/>
       <c r="B545" s="3"/>
     </row>
     <row r="546" spans="1:3">
@@ -27281,42 +27264,42 @@
       </c>
     </row>
     <row r="548" spans="1:3">
-      <c r="A548" s="35">
-        <v>1</v>
-      </c>
-      <c r="B548" s="35" t="s">
+      <c r="A548" s="34">
+        <v>1</v>
+      </c>
+      <c r="B548" s="34" t="s">
         <v>1137</v>
       </c>
     </row>
     <row r="549" spans="1:3">
-      <c r="A549" s="35">
+      <c r="A549" s="34">
         <v>2</v>
       </c>
-      <c r="B549" s="35" t="s">
+      <c r="B549" s="34" t="s">
         <v>1251</v>
       </c>
     </row>
     <row r="550" spans="1:3">
-      <c r="A550" s="35">
+      <c r="A550" s="34">
         <v>3</v>
       </c>
-      <c r="B550" s="35" t="s">
+      <c r="B550" s="34" t="s">
         <v>1252</v>
       </c>
     </row>
     <row r="551" spans="1:3">
-      <c r="A551" s="35">
+      <c r="A551" s="34">
         <v>4</v>
       </c>
-      <c r="B551" s="35" t="s">
+      <c r="B551" s="34" t="s">
         <v>1253</v>
       </c>
     </row>
     <row r="552" spans="1:3">
-      <c r="A552" s="35">
+      <c r="A552" s="34">
         <v>5</v>
       </c>
-      <c r="B552" s="35" t="s">
+      <c r="B552" s="34" t="s">
         <v>1133</v>
       </c>
     </row>
@@ -27329,7 +27312,7 @@
       </c>
     </row>
     <row r="554" spans="1:3">
-      <c r="A554" s="30"/>
+      <c r="A554" s="29"/>
       <c r="B554" s="3"/>
     </row>
     <row r="555" spans="1:3">
@@ -27350,42 +27333,42 @@
       </c>
     </row>
     <row r="557" spans="1:3">
-      <c r="A557" s="35">
-        <v>1</v>
-      </c>
-      <c r="B557" s="35" t="s">
+      <c r="A557" s="34">
+        <v>1</v>
+      </c>
+      <c r="B557" s="34" t="s">
         <v>1254</v>
       </c>
     </row>
     <row r="558" spans="1:3">
-      <c r="A558" s="35">
+      <c r="A558" s="34">
         <v>2</v>
       </c>
-      <c r="B558" s="35" t="s">
+      <c r="B558" s="34" t="s">
         <v>1255</v>
       </c>
     </row>
     <row r="559" spans="1:3">
-      <c r="A559" s="35">
+      <c r="A559" s="34">
         <v>3</v>
       </c>
-      <c r="B559" s="35" t="s">
+      <c r="B559" s="34" t="s">
         <v>1256</v>
       </c>
     </row>
     <row r="560" spans="1:3">
-      <c r="A560" s="35">
+      <c r="A560" s="34">
         <v>4</v>
       </c>
-      <c r="B560" s="35" t="s">
+      <c r="B560" s="34" t="s">
         <v>1257</v>
       </c>
     </row>
     <row r="561" spans="1:3">
-      <c r="A561" s="35">
+      <c r="A561" s="34">
         <v>5</v>
       </c>
-      <c r="B561" s="35" t="s">
+      <c r="B561" s="34" t="s">
         <v>1258</v>
       </c>
     </row>
@@ -27497,7 +27480,7 @@
       <c r="A577" s="6" t="s">
         <v>962</v>
       </c>
-      <c r="C577" s="8" t="s">
+      <c r="C577" s="39" t="s">
         <v>961</v>
       </c>
     </row>
@@ -27582,18 +27565,18 @@
       </c>
     </row>
     <row r="589" spans="1:3">
-      <c r="A589" s="33">
-        <v>1</v>
-      </c>
-      <c r="B589" s="32" t="s">
+      <c r="A589" s="32">
+        <v>1</v>
+      </c>
+      <c r="B589" s="31" t="s">
         <v>1270</v>
       </c>
     </row>
     <row r="590" spans="1:3">
-      <c r="A590" s="33">
+      <c r="A590" s="32">
         <v>2</v>
       </c>
-      <c r="B590" s="32" t="s">
+      <c r="B590" s="31" t="s">
         <v>1271</v>
       </c>
     </row>
@@ -27606,7 +27589,7 @@
       </c>
     </row>
     <row r="592" spans="1:3">
-      <c r="A592" s="33">
+      <c r="A592" s="32">
         <v>4</v>
       </c>
       <c r="B592" s="7" t="s">
@@ -27614,7 +27597,7 @@
       </c>
     </row>
     <row r="593" spans="1:3">
-      <c r="A593" s="33">
+      <c r="A593" s="32">
         <v>9</v>
       </c>
       <c r="B593" s="7" t="s">
@@ -27622,7 +27605,7 @@
       </c>
     </row>
     <row r="594" spans="1:3">
-      <c r="A594" s="33"/>
+      <c r="A594" s="32"/>
     </row>
     <row r="595" spans="1:3">
       <c r="A595" s="41" t="s">
@@ -27642,7 +27625,7 @@
       </c>
     </row>
     <row r="597" spans="1:3">
-      <c r="A597" s="33">
+      <c r="A597" s="32">
         <v>1</v>
       </c>
       <c r="B597" s="3" t="s">
@@ -27650,7 +27633,7 @@
       </c>
     </row>
     <row r="598" spans="1:3">
-      <c r="A598" s="33">
+      <c r="A598" s="32">
         <v>2</v>
       </c>
       <c r="B598" s="22" t="s">
@@ -27658,7 +27641,7 @@
       </c>
     </row>
     <row r="599" spans="1:3">
-      <c r="A599" s="33">
+      <c r="A599" s="32">
         <v>3</v>
       </c>
       <c r="B599" s="22" t="s">
@@ -27666,7 +27649,7 @@
       </c>
     </row>
     <row r="600" spans="1:3">
-      <c r="A600" s="33">
+      <c r="A600" s="32">
         <v>4</v>
       </c>
       <c r="B600" s="22" t="s">
@@ -27674,7 +27657,7 @@
       </c>
     </row>
     <row r="601" spans="1:3">
-      <c r="A601" s="33">
+      <c r="A601" s="32">
         <v>5</v>
       </c>
       <c r="B601" s="22" t="s">
@@ -27682,7 +27665,7 @@
       </c>
     </row>
     <row r="602" spans="1:3">
-      <c r="A602" s="33">
+      <c r="A602" s="32">
         <v>9</v>
       </c>
       <c r="B602" s="22" t="s">
@@ -27706,10 +27689,10 @@
       </c>
     </row>
     <row r="606" spans="1:3">
-      <c r="A606" s="33">
-        <v>1</v>
-      </c>
-      <c r="B606" s="33" t="s">
+      <c r="A606" s="32">
+        <v>1</v>
+      </c>
+      <c r="B606" s="32" t="s">
         <v>1278</v>
       </c>
     </row>
@@ -27730,7 +27713,7 @@
       </c>
     </row>
     <row r="609" spans="1:2">
-      <c r="A609" s="33">
+      <c r="A609" s="32">
         <v>9</v>
       </c>
       <c r="B609" s="22" t="s">

</xml_diff>